<commit_message>
Re-acquire the 15 approved datasets, verify them, and add the E2-E4/E7 runners
All 15 approved files downloaded again (PhysioNet and OpenML via their www
hosts, which the network policy allows). Validation now checks PhysioNet
zips member by member against SHA256SUMS.txt, parses WFDB records and
multi-table archives, and scopes each parse config to the file it
describes. Nine tabular datasets pass the leakage-aware preprocessing check;
CLN-006 still fails to parse because UCI ships it as a .rar inside the zip.

New hcds.experiments runs E2-E4 on identical (grouped where needed) folds
with Nadeau-Bengio corrected t-tests; hcds.ecg runs E7 on the MIT-BIH
inter-patient split. IQP kernel states are now computed directly with numpy
(matches PennyLane to 1e-15, tested). E2 and E3 results included.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014qao7kdbjq3a44H4ZxKhmq
</commit_message>
<xml_diff>
--- a/healthcare-datasets/catalog/master_catalog.xlsx
+++ b/healthcare-datasets/catalog/master_catalog.xlsx
@@ -33,7 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Source registry'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Access restrictions'!$A$1:$H$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'QML feasibility'!$A$1:$W$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Acquisition manifest'!$A$1:$M$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Acquisition manifest'!$A$1:$M$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Overlaps &amp; mirrors'!$A$1:$C$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,13 +43,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -60,7 +63,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -68,12 +71,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,107 +455,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -2782,7 +2794,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -2889,7 +2901,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
@@ -2996,7 +3008,7 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
@@ -3210,7 +3222,7 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -3317,7 +3329,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Integrity verified</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
@@ -3424,7 +3436,7 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
@@ -3531,7 +3543,7 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
@@ -3745,7 +3757,7 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
@@ -3852,7 +3864,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -4066,7 +4078,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -11021,7 +11033,7 @@
       </c>
       <c r="S99" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T99" t="inlineStr">
@@ -11877,7 +11889,7 @@
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T107" t="inlineStr">
@@ -12733,7 +12745,7 @@
       </c>
       <c r="S115" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T115" t="inlineStr">
@@ -13054,7 +13066,7 @@
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13084,42 +13096,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>access_level</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>license</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>canonical_url</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>next_step</t>
         </is>
@@ -14485,117 +14497,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>task</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>n_samples_used</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>n_features_raw</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>size_basis</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>label_structure</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>class_imbalance</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>reduction</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>reduced_features</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>angle_qubits</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>amplitude_qubits</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>amplitude_state_prep_cnots</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>basis_qubits</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>zz_feature_map_entanglers</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>qsvm_kernel_evals_full</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>qsvm_max_train_samples</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>simulator_tier</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>recommended_encoding</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>recommended_qml_models</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>classical_baselines</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>qml_suitability</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>trainability_notes</t>
         </is>
@@ -16165,71 +16177,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>acquisition_method</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>requested_files</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>local_path</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>download_status</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>timestamp_utc</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>file_size_bytes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>expected_checksum</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>error_or_reason</t>
         </is>
@@ -17057,8 +17069,1773 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CLN-009</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/17/breast+cancer+wisconsin+diagnostic.zip</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>breast_cancer_wisconsin_diagnostic.zip</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>clinical_tabular/cancer/raw/CLN-009/breast_cancer_wisconsin_diagnostic.zip</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:47:33Z</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>51284</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>bc154869ef13f753f9e2b5a17e248cfe1ba4b6721db7c4da9f4880e40b05d3af</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CLN-001</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/45/data.csv</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>heart_disease_data.csv</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>clinical_tabular/cardiovascular/raw/CLN-001/heart_disease_data.csv</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:47:34Z</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>11334</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>868cd646a53ffbc55611192bae7496911a163937c185710f6b8aa11549b88df1</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CLN-002</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://openml.org/data/v1/download/37/diabetes.arff</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>diabetes_openml37.arff</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>clinical_tabular/diabetes/raw/CLN-002/diabetes_openml37.arff</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:47:36Z</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>1 (uploaded 2014-04-06; status active)</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>md5:3cbaa3e54586aa88cf6aacb4033e4470</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CLN-003</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/296/diabetes+130-us+hospitals+for+years+1999-2008.zip</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>diabetes_130_us_hospitals.zip</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>clinical_tabular/diabetes/raw/CLN-003/diabetes_130_us_hospitals.zip</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:48:12Z</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>3170254</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>f82ac129da2ddd2299391ff6fbae3a6a58b3edcf59ac9d7bd480c00fe453112a</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CLN-005</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/529/early+stage+diabetes+risk+prediction+dataset.zip</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>early_stage_diabetes.zip</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>clinical_tabular/diabetes/raw/CLN-005/early_stage_diabetes.zip</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:48:14Z</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>34828</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>67594c0f11257688b57493798e70737b7156ba37a2e6ac75507ae3a35221a388</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CLN-006</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/336/chronic+kidney+disease.zip</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>chronic_kidney_disease.zip</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>clinical_tabular/kidney/raw/CLN-006/chronic_kidney_disease.zip</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:48:15Z</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>19410</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>3f0d0e5bab0f453165acfa2c77eae695393089c5b338cb4cd98339c96a26a585</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CLN-007</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/225/ilpd+indian+liver+patient+dataset.zip</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ilpd.zip</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>clinical_tabular/liver/raw/CLN-007/ilpd.zip</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:48:17Z</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>23931</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>60e18fbfe7f84daf58c178ea280ba5fe8db7e2507aabce01b57425b3b822cf0b</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CLN-008</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/571/hcv+data.zip</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>hcv_data.zip</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>clinical_tabular/liver/raw/CLN-008/hcv_data.zip</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:48:19Z</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>46303</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>0fafa2c4ae94db98b95f35cd41e9f4cedbd1e105282ab0cd7b5ed3effe5a05d8</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CLN-010</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/519/heart+failure+clinical+records.zip</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>heart_failure_clinical_records.zip</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>clinical_tabular/cardiovascular/raw/CLN-010/heart_failure_clinical_records.zip</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:48:21Z</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>12421</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>f0739603e2f9573ffc7d509573cbf9bcb4cc889e4eea0f35a75bec68fc9163d7</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CLN-011</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/383/cervical+cancer+risk+factors.zip</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>cervical_cancer_risk_factors.zip</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>clinical_tabular/cancer/raw/CLN-011/cervical_cancer_risk_factors.zip</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:48:24Z</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>102221</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>d86f38fbb1f4c40c22c240127875d7a83a2f96238f7ed5a388e2277cfb79a742</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CLN-013</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://physionet.org/content/mimic-iv-demo/get-zip/2.2/</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>None; conform to license</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>mimic_iv_demo_2.2.zip</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>clinical_tabular/icu/raw/CLN-013/mimic_iv_demo_2.2.zip</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:48:25Z</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2.2 (published January 31, 2023)</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>16189661</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>97301a03820e8f41af211cf3462ddc19aefe75bbed05f11753859affaafeb8ec</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TS-001</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://physionet.org/content/mitdb/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>mitdb_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>time_series/ecg/raw/TS-001/mitdb_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:50:02Z</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>77030320</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>47b26926927c11bd9174154d367c811afc1b186f650f8a205931ca8c520f0a87</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TS-009</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://physionet.org/content/bidmc/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>bidmc_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>time_series/spo2/raw/TS-009/bidmc_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:58:01Z</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>217902224</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>7c09847e8b9c9ad0005ad6f4041e887119e2ad9a745b6a63b1b394bd439f693b</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TS-017</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://physionet.org/content/noneeg/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>noneeg_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>time_series/wearable/raw/TS-017/noneeg_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:20:06Z</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>3925168</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>6700b0f78f3e2724d9049a3398f9294dc7b15b296284326e13b639bc1792096e</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TS-020</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://physionet.org/content/wearable-exam-stress/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>wearable_exam_stress_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>time_series/wearable/raw/TS-020/wearable_exam_stress_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:20:31Z</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>1.0.0 (latest)</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>85968624</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>f9c0e488054d8653ba7c69177891359016ffc4b4946b376b022ce864bc257e58</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>CLN-009</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>sklearn://datasets/data/breast_cancer.csv</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>sklearn_bundled (scikit-learn 1.9.1 package data)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>breast_cancer_sklearn_copy.csv</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>clinical_tabular/cancer/raw/CLN-009/breast_cancer_sklearn_copy.csv</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:53:56Z</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>119913</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>fed3eb72d0575ef6192293f5093c6e801b1476b577d0386bf4455504522172ed</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>CLN-009</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/17/breast+cancer+wisconsin+diagnostic.zip</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>breast_cancer_wisconsin_diagnostic.zip</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>clinical_tabular/cancer/raw/CLN-009/breast_cancer_wisconsin_diagnostic.zip</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:53:57Z</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>51284</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>bc154869ef13f753f9e2b5a17e248cfe1ba4b6721db7c4da9f4880e40b05d3af</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>CLN-001</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/45/data.csv</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>heart_disease_data.csv</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>clinical_tabular/cardiovascular/raw/CLN-001/heart_disease_data.csv</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:53:58Z</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>11334</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>868cd646a53ffbc55611192bae7496911a163937c185710f6b8aa11549b88df1</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>CLN-002</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://www.openml.org/data/v1/download/37/diabetes.arff</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>diabetes_openml37.arff</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>clinical_tabular/diabetes/raw/CLN-002/diabetes_openml37.arff</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:54:00Z</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>1 (uploaded 2014-04-06; status active)</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>37419</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>4eddd5b2b64679e8888348e306520a393d6a28e1ddc9643cfb76fc5d912d6d40</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>md5:3cbaa3e54586aa88cf6aacb4033e4470</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CLN-003</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/296/diabetes+130-us+hospitals+for+years+1999-2008.zip</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>diabetes_130_us_hospitals.zip</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>clinical_tabular/diabetes/raw/CLN-003/diabetes_130_us_hospitals.zip</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:54:02Z</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>3170254</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>f82ac129da2ddd2299391ff6fbae3a6a58b3edcf59ac9d7bd480c00fe453112a</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>CLN-005</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/529/early+stage+diabetes+risk+prediction+dataset.zip</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>early_stage_diabetes.zip</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>clinical_tabular/diabetes/raw/CLN-005/early_stage_diabetes.zip</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:54:04Z</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>34828</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>67594c0f11257688b57493798e70737b7156ba37a2e6ac75507ae3a35221a388</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>CLN-006</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/336/chronic+kidney+disease.zip</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>chronic_kidney_disease.zip</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>clinical_tabular/kidney/raw/CLN-006/chronic_kidney_disease.zip</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:54:06Z</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>19410</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>3f0d0e5bab0f453165acfa2c77eae695393089c5b338cb4cd98339c96a26a585</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>CLN-007</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/225/ilpd+indian+liver+patient+dataset.zip</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ilpd.zip</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>clinical_tabular/liver/raw/CLN-007/ilpd.zip</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:54:08Z</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>23931</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>60e18fbfe7f84daf58c178ea280ba5fe8db7e2507aabce01b57425b3b822cf0b</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CLN-008</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/571/hcv+data.zip</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>hcv_data.zip</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>clinical_tabular/liver/raw/CLN-008/hcv_data.zip</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:54:10Z</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>46303</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>0fafa2c4ae94db98b95f35cd41e9f4cedbd1e105282ab0cd7b5ed3effe5a05d8</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>CLN-010</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/519/heart+failure+clinical+records.zip</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>heart_failure_clinical_records.zip</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>clinical_tabular/cardiovascular/raw/CLN-010/heart_failure_clinical_records.zip</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:54:12Z</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>12421</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>f0739603e2f9573ffc7d509573cbf9bcb4cc889e4eea0f35a75bec68fc9163d7</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>CLN-011</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/383/cervical+cancer+risk+factors.zip</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>None (no login)</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>cervical_cancer_risk_factors.zip</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>clinical_tabular/cancer/raw/CLN-011/cervical_cancer_risk_factors.zip</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:54:14Z</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>102221</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>d86f38fbb1f4c40c22c240127875d7a83a2f96238f7ed5a388e2277cfb79a742</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CLN-013</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/mimic-iv-demo/get-zip/2.2/</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>None; conform to license</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>mimic_iv_demo_2.2.zip</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>clinical_tabular/icu/raw/CLN-013/mimic_iv_demo_2.2.zip</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:54:16Z</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2.2 (published January 31, 2023)</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>16189661</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>97301a03820e8f41af211cf3462ddc19aefe75bbed05f11753859affaafeb8ec</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>TS-001</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/mitdb/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>mitdb_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>time_series/ecg/raw/TS-001/mitdb_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:55:53Z</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>77030320</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>47b26926927c11bd9174154d367c811afc1b186f650f8a205931ca8c520f0a87</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>TS-009</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/bidmc/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>bidmc_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>time_series/spo2/raw/TS-009/bidmc_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-10-04T11:03:15Z</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>217902224</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>7c09847e8b9c9ad0005ad6f4041e887119e2ad9a745b6a63b1b394bd439f693b</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>TS-017</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/noneeg/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>noneeg_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>time_series/wearable/raw/TS-017/noneeg_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-10-04T11:25:00Z</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>3925168</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>6700b0f78f3e2724d9049a3398f9294dc7b15b296284326e13b639bc1792096e</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>TS-020</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/wearable-exam-stress/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>wearable_exam_stress_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>time_series/wearable/raw/TS-020/wearable_exam_stress_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2026-10-04T11:34:08Z</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>1.0.0 (latest)</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>85968624</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>f9c0e488054d8653ba7c69177891359016ffc4b4946b376b022ce864bc257e58</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M17"/>
+  <autoFilter ref="A1:M48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17073,17 +18850,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id_a</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>dataset_id_b</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
@@ -17819,107 +19596,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -20081,107 +21858,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -20280,7 +22057,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -20387,7 +22164,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -20494,7 +22271,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -20708,7 +22485,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -20815,7 +22592,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Integrity verified</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -20922,7 +22699,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -21029,7 +22806,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -21243,7 +23020,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -21350,7 +23127,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -21564,7 +23341,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -22450,107 +24227,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -24712,107 +26489,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -24911,7 +26688,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -25767,7 +27544,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -26623,7 +28400,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -26944,7 +28721,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -26974,107 +28751,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -29022,107 +30799,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -31070,177 +32847,177 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>canonical_url</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>download_or_api_url</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>doi</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>application</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>modality</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>file_formats</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>sample_count</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>subject_count</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>feature_count</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>target</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>class_distribution</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>geographic_coverage</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>temporal_coverage</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>collection_method</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>missing_data</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>annotation</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>license</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>access_level</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>download_method</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>citation</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>checksum_or_manifest</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>limitations</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>mirrors</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>verification_status</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>derived_status</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>verification_method</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>approx_size</t>
         </is>
@@ -34944,7 +36721,7 @@
       </c>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="AG22" t="inlineStr">
@@ -35121,7 +36898,7 @@
       </c>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="AG23" t="inlineStr">
@@ -35298,7 +37075,7 @@
       </c>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="AG24" t="inlineStr">
@@ -35652,7 +37429,7 @@
       </c>
       <c r="AF26" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="AG26" t="inlineStr">
@@ -35829,7 +37606,7 @@
       </c>
       <c r="AF27" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Integrity verified</t>
         </is>
       </c>
       <c r="AG27" t="inlineStr">
@@ -36006,7 +37783,7 @@
       </c>
       <c r="AF28" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="AG28" t="inlineStr">
@@ -36183,7 +37960,7 @@
       </c>
       <c r="AF29" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="AG29" t="inlineStr">
@@ -36537,7 +38314,7 @@
       </c>
       <c r="AF31" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="AG31" t="inlineStr">
@@ -36714,7 +38491,7 @@
       </c>
       <c r="AF32" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="AG32" t="inlineStr">
@@ -37068,7 +38845,7 @@
       </c>
       <c r="AF34" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG34" t="inlineStr">
@@ -48573,7 +50350,7 @@
       </c>
       <c r="AF99" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG99" t="inlineStr">
@@ -49989,7 +51766,7 @@
       </c>
       <c r="AF107" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG107" t="inlineStr">
@@ -51405,7 +53182,7 @@
       </c>
       <c r="AF115" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG115" t="inlineStr">
@@ -51936,7 +53713,7 @@
       </c>
       <c r="AF118" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG118" t="inlineStr">
@@ -51971,42 +53748,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>programmatic_access</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>access_model</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>search_method</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>container_reachable_2026_10_04</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>datasets_in_catalogue</t>
         </is>

</xml_diff>

<commit_message>
Approve batch-2 downloads; acquire and parse PubMedQA (NLP-005)
Adds 13 open, clearly licensed datasets to the acquisition plan (UCI gene
sequences and RNA-seq, PhysioNet ECG/EEG/sepsis, CDC, OWID, World Bank,
PubMedQA). PubMedQA is downloaded, integrity-checked and parsed here; the
rest need a session whose network reaches those hosts. read_tabular gains
a JSON reader and profile() counts duplicates on list-valued cells.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01223oBQ9XyB8ZKp9WFb8NAF
</commit_message>
<xml_diff>
--- a/healthcare-datasets/catalog/master_catalog.xlsx
+++ b/healthcare-datasets/catalog/master_catalog.xlsx
@@ -33,7 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Source registry'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Access restrictions'!$A$1:$H$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'QML feasibility'!$A$1:$W$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Acquisition manifest'!$A$1:$M$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Acquisition manifest'!$A$1:$M$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Overlaps &amp; mirrors'!$A$1:$C$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,16 +43,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -63,7 +60,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -71,21 +68,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -455,107 +443,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -5469,7 +5457,7 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
@@ -13096,42 +13084,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>access_level</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>license</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>canonical_url</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>next_step</t>
         </is>
@@ -14497,117 +14485,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>task</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>n_samples_used</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>n_features_raw</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>size_basis</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>label_structure</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>class_imbalance</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>reduction</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>reduced_features</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>angle_qubits</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>amplitude_qubits</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>amplitude_state_prep_cnots</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>basis_qubits</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>zz_feature_map_entanglers</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>qsvm_kernel_evals_full</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>qsvm_max_train_samples</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>simulator_tier</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>recommended_encoding</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>recommended_qml_models</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>classical_baselines</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>qml_suitability</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>trainability_notes</t>
         </is>
@@ -16177,71 +16165,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>acquisition_method</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>requested_files</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>local_path</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>download_status</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>timestamp_utc</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>file_size_bytes</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>expected_checksum</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>error_or_reason</t>
         </is>
@@ -18834,8 +18822,61 @@
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>NLP-005</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/pubmedqa/pubmedqa/master/data/ori_pqal.json</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>pubmedqa_pqal.json</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>healthcare_nlp/medical_qa/raw/NLP-005/pubmedqa_pqal.json</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:32:52Z</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>2584787</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>8b3276be8942ebbd77f3ddcda12c1749bf0e490045a736fd8438ee40cf37a41d</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M48"/>
+  <autoFilter ref="A1:M49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18850,17 +18891,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dataset_id_a</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>dataset_id_b</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
@@ -19596,107 +19637,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -21858,107 +21899,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -24227,107 +24268,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -26489,107 +26530,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -28751,107 +28792,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -30799,107 +30840,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -31426,7 +31467,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -32847,177 +32888,177 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>canonical_url</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>download_or_api_url</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>doi</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>application</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>modality</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>file_formats</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>sample_count</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>subject_count</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>feature_count</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>target</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>class_distribution</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>geographic_coverage</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>temporal_coverage</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>collection_method</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>missing_data</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>annotation</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>license</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>access_level</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>download_method</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>citation</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>checksum_or_manifest</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>limitations</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>mirrors</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>verification_status</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>derived_status</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>verification_method</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>approx_size</t>
         </is>
@@ -41146,7 +41187,7 @@
       </c>
       <c r="AF47" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG47" t="inlineStr">
@@ -53748,42 +53789,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>programmatic_access</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>access_model</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>search_method</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>container_reachable_2026_10_04</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>datasets_in_catalogue</t>
         </is>

</xml_diff>

<commit_message>
Acquire batch-2 UCI sets, run E5 on BIO-003, record blocked public-health hosts
BIO-001/002/003 downloaded from UCI and validated; BIO-001/002 get parse
configs, and archive parsing now reads a .tar.gz inside a zip (BIO-003).
New hcds.rnaseq runs E5: classical models reach ~0.999 accuracy, the
one-vs-rest VQC 0.970 and the IQP QSVM 0.921. data.cdc.gov,
catalog.ourworldindata.org and api.worldbank.org are blocked by the
network policy (PH-008/009/014/015); PhysioNet offers no zip for TS-019.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01233dsRAwyA6Arys3vibR2G
</commit_message>
<xml_diff>
--- a/healthcare-datasets/catalog/master_catalog.xlsx
+++ b/healthcare-datasets/catalog/master_catalog.xlsx
@@ -33,7 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Source registry'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Access restrictions'!$A$1:$H$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'QML feasibility'!$A$1:$W$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Acquisition manifest'!$A$1:$M$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Acquisition manifest'!$A$1:$M$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Overlaps &amp; mirrors'!$A$1:$C$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,13 +43,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -60,7 +63,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -68,12 +71,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,107 +455,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -642,7 +654,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -749,7 +761,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -856,7 +868,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -13084,42 +13096,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>access_level</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>license</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>canonical_url</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>next_step</t>
         </is>
@@ -14485,117 +14497,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>task</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>n_samples_used</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>n_features_raw</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>size_basis</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>label_structure</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>class_imbalance</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>reduction</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>reduced_features</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>angle_qubits</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>amplitude_qubits</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>amplitude_state_prep_cnots</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>basis_qubits</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>zz_feature_map_entanglers</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>qsvm_kernel_evals_full</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>qsvm_max_train_samples</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>simulator_tier</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>recommended_encoding</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>recommended_qml_models</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>classical_baselines</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>qml_suitability</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>trainability_notes</t>
         </is>
@@ -16165,71 +16177,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>acquisition_method</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>requested_files</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>local_path</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>download_status</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>timestamp_utc</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>file_size_bytes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>expected_checksum</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>error_or_reason</t>
         </is>
@@ -18875,8 +18887,426 @@
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BIO-001</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/69/molecular+biology+splice+junction+gene+sequences.zip</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>splice_junction.zip</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>biomedical/genomics/raw/BIO-001/splice_junction.zip</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:35:41Z</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Donated 1991-12-31</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>167041</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>3e7ce5dcbeec8c221f57dda495611b9d6ec9525551f445419f5c74cc38067e4e</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>BIO-002</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/67/molecular+biology+promoter+gene+sequences.zip</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>promoter_sequences.zip</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>biomedical/genomics/raw/BIO-002/promoter_sequences.zip</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:35:42Z</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Donated 1990-06-29</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>5237</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>56d462fe7e27dfece24dd5033e2c359c604b5675f5ba448eb0a9ceb7284b4eb2</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>BIO-003</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://archive.ics.uci.edu/static/public/401/gene+expression+cancer+rna+seq.zip</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>gene_expression_cancer_rnaseq.zip</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>biomedical/transcriptomics/raw/BIO-003/gene_expression_cancer_rnaseq.zip</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:35:44Z</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Donated 2016-06-08</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>72856486</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>06bbb28393ed85b4365f461f20ad75996f2579af4a047945c038ec27386e3bfb</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TS-019</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/challenge-2019/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>challenge_2019_sepsis.zip</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>time_series/icu_vitals/raw/TS-019/challenge_2019_sepsis.zip</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:35:48Z</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>HTTPError: HTTP Error 404: Not Found</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>PH-009</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://data.cdc.gov/api/views/bi63-dtpu/rows.csv?&lt;redacted&gt;</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>nchs_leading_causes_of_death.csv</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>public_health/mortality/raw/PH-009/nchs_leading_causes_of_death.csv</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:39:19Z</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Rows updated 2019-10-24</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>PH-008</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://data.cdc.gov/api/views/swc5-untb/rows.csv?&lt;redacted&gt;</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>places_county_2025.csv</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>public_health/epidemiology/raw/PH-008/places_county_2025.csv</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:39:50Z</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2025 release</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>PH-014</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://catalog.ourworldindata.org/garden/covid/latest/compact/compact.csv</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>owid_covid_compact.csv</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>public_health/epidemiology/raw/PH-014/owid_covid_compact.csv</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:40:23Z</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Archived; last update 19 August 2024</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>PH-015</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://api.worldbank.org/v2/en/topic/8?&lt;redacted&gt;</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>wdi_health_topic.zip</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>public_health/social_determinants/raw/PH-015/wdi_health_topic.zip</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:40:56Z</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Updated 2025-12-19</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt;</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M49"/>
+  <autoFilter ref="A1:M57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18891,17 +19321,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id_a</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>dataset_id_b</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
@@ -19637,107 +20067,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -21899,107 +22329,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -24268,107 +24698,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -24467,7 +24897,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -24574,7 +25004,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -24681,7 +25111,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -26530,107 +26960,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -28792,107 +29222,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -30840,107 +31270,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -32888,177 +33318,177 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>canonical_url</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>download_or_api_url</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>doi</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>application</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>modality</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>file_formats</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>sample_count</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>subject_count</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>feature_count</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>target</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>class_distribution</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>geographic_coverage</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>temporal_coverage</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>collection_method</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>missing_data</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>annotation</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>license</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>access_level</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>download_method</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>citation</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>checksum_or_manifest</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>limitations</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>mirrors</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>verification_status</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>derived_status</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>verification_method</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>approx_size</t>
         </is>
@@ -33222,7 +33652,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -33399,7 +33829,7 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Preprocessing validated</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
@@ -33576,7 +34006,7 @@
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
@@ -53789,42 +54219,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>programmatic_access</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>access_model</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>search_method</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>container_reachable_2026_10_04</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>datasets_in_catalogue</t>
         </is>

</xml_diff>

<commit_message>
Acquire PH-014 (OWID COVID) via GitHub mirror; catalogue.ourworldindata.org still blocked
PH-008/009 (data.cdc.gov), PH-015 (api.worldbank.org) and the Snowflake
account host remain denied by network policy; Snowflake env vars are not
set in this environment.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RFHETRrgnvYKbVqZnx6qRu
</commit_message>
<xml_diff>
--- a/healthcare-datasets/catalog/master_catalog.xlsx
+++ b/healthcare-datasets/catalog/master_catalog.xlsx
@@ -33,7 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Source registry'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Access restrictions'!$A$1:$H$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'QML feasibility'!$A$1:$W$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Acquisition manifest'!$A$1:$M$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Acquisition manifest'!$A$1:$M$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Overlaps &amp; mirrors'!$A$1:$C$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,16 +43,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -63,7 +60,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -71,21 +68,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -455,107 +443,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -10498,7 +10486,7 @@
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T94" t="inlineStr">
@@ -13096,42 +13084,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>access_level</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>license</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>canonical_url</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>next_step</t>
         </is>
@@ -14497,117 +14485,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>task</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>n_samples_used</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>n_features_raw</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>size_basis</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>label_structure</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>class_imbalance</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>reduction</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>reduced_features</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>angle_qubits</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>amplitude_qubits</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>amplitude_state_prep_cnots</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>basis_qubits</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>zz_feature_map_entanglers</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>qsvm_kernel_evals_full</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>qsvm_max_train_samples</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>simulator_tier</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>recommended_encoding</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>recommended_qml_models</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>classical_baselines</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>qml_suitability</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>trainability_notes</t>
         </is>
@@ -16177,71 +16165,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:M58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>acquisition_method</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>requested_files</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>local_path</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>download_status</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>timestamp_utc</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>file_size_bytes</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>expected_checksum</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>error_or_reason</t>
         </is>
@@ -19305,8 +19293,61 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>PH-014</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/owid/covid-19-data/master/public/data/owid-covid-data.csv</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>owid-covid-data.csv</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>public_health/epidemiology/raw/PH-014/owid-covid-data.csv</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>2026-10-04T17:24:45Z</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Archived; last update 19 August 2024</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>97714880</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>fa4423a904ce1b12a9b01ad6cf0e7c535a3dacee435fd96ba41975f1fae089fc</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M57"/>
+  <autoFilter ref="A1:M58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19321,17 +19362,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dataset_id_a</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>dataset_id_b</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
@@ -20067,107 +20108,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -22329,107 +22370,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -24698,107 +24739,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -26960,107 +27001,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -29222,107 +29263,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -30812,7 +30853,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -31270,107 +31311,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -33318,177 +33359,177 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>subcategory</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>canonical_url</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>download_or_api_url</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>doi</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>application</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>modality</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>file_formats</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>sample_count</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>subject_count</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>feature_count</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>target</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>class_distribution</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>geographic_coverage</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>temporal_coverage</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>collection_method</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>missing_data</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>annotation</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>license</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>access_level</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>download_method</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>citation</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>checksum_or_manifest</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>limitations</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>mirrors</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>verification_status</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>derived_status</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>verification_method</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>approx_size</t>
         </is>
@@ -49936,7 +49977,7 @@
       </c>
       <c r="AF94" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG94" t="inlineStr">
@@ -54219,42 +54260,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>programmatic_access</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>access_model</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>search_method</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>container_reachable_2026_10_04</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>datasets_in_catalogue</t>
         </is>

</xml_diff>

<commit_message>
Acquire PH-008, PH-009 and PH-015; parse World Bank CSV preamble
data.cdc.gov and api.worldbank.org are reachable in this environment, so the
three public-health downloads now succeed. World Bank bulk CSVs carry two
metadata lines above the header; parse_archive_tables now skips them.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtBZjWU66ytZWo1vzz3oXx
</commit_message>
<xml_diff>
--- a/healthcare-datasets/catalog/master_catalog.xlsx
+++ b/healthcare-datasets/catalog/master_catalog.xlsx
@@ -33,7 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Source registry'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Access restrictions'!$A$1:$H$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'QML feasibility'!$A$1:$W$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Acquisition manifest'!$A$1:$M$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Acquisition manifest'!$A$1:$M$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Overlaps &amp; mirrors'!$A$1:$C$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,13 +43,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -60,7 +63,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -68,12 +71,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,107 +455,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -9844,7 +9856,7 @@
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T88" t="inlineStr">
@@ -9951,7 +9963,7 @@
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T89" t="inlineStr">
@@ -10593,7 +10605,7 @@
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T95" t="inlineStr">
@@ -13084,42 +13096,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>access_level</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>license</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>canonical_url</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>next_step</t>
         </is>
@@ -14485,117 +14497,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>task</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>n_samples_used</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>n_features_raw</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>size_basis</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>label_structure</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>class_imbalance</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>reduction</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>reduced_features</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>angle_qubits</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>amplitude_qubits</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>amplitude_state_prep_cnots</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>basis_qubits</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>zz_feature_map_entanglers</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>qsvm_kernel_evals_full</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>qsvm_max_train_samples</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>simulator_tier</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>recommended_encoding</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>recommended_qml_models</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>classical_baselines</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>qml_suitability</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>trainability_notes</t>
         </is>
@@ -16165,71 +16177,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M58"/>
+  <dimension ref="A1:M62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>acquisition_method</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>requested_files</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>local_path</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>download_status</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>timestamp_utc</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>file_size_bytes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>expected_checksum</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>error_or_reason</t>
         </is>
@@ -19346,8 +19358,220 @@
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>PH-009</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://data.cdc.gov/api/views/bi63-dtpu/rows.csv?&lt;redacted&gt;</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>nchs_leading_causes_of_death.csv</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>public_health/mortality/raw/PH-009/nchs_leading_causes_of_death.csv</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>2026-10-04T18:09:18Z</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Rows updated 2019-10-24</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>842709</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>1971e6664c76457a5c32e4c86aa103ba404b7be5d17ddb6e6dfc0075479c85d9</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>PH-008</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://data.cdc.gov/api/views/swc5-untb/rows.csv?&lt;redacted&gt;</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>places_county_2025.csv</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>public_health/epidemiology/raw/PH-008/places_county_2025.csv</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2026-10-04T18:09:19Z</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>2025 release</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>53396904</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>2dc8d4ae93543a217973bdc2d774855134ca01d8adf00c77a082acc4b8ce3377</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>PH-015</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://api.worldbank.org/v2/en/topic/8?&lt;redacted&gt;</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>wdi_health_topic.zip</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>public_health/social_determinants/raw/PH-015/wdi_health_topic.zip</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2026-10-04T18:10:10Z</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Updated 2025-12-19</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>13735212</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>8e7e4b96054197b2009203c3494363603522d0a59c2c51f4df8edda24846bd06</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>PH-015</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://api.worldbank.org/v2/en/topic/8?&lt;redacted&gt;</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>wdi_health_topic.zip</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>public_health/social_determinants/raw/PH-015/wdi_health_topic.zip</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2026-10-04T18:11:17Z</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Updated 2025-12-19</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
+        <v>13735212</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>8e7e4b96054197b2009203c3494363603522d0a59c2c51f4df8edda24846bd06</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M58"/>
+  <autoFilter ref="A1:M62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19362,17 +19586,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id_a</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>dataset_id_b</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
@@ -20108,107 +20332,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -22370,107 +22594,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -24739,107 +24963,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -27001,107 +27225,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -29263,107 +29487,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -30211,7 +30435,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -30318,7 +30542,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -30960,7 +31184,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -31311,107 +31535,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Canonical URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sample Count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature Count</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File Format</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Access Requirements</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Download Method</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dataset Version</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Classical ML Suitability</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>QML Suitability</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -33359,177 +33583,177 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>dataset_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>canonical_url</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>download_or_api_url</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>doi</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>application</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>modality</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>file_formats</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>sample_count</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>subject_count</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>feature_count</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>target</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>class_distribution</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>geographic_coverage</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>temporal_coverage</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>collection_method</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>missing_data</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>annotation</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>license</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>access_level</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>access_prerequisites</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>download_method</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>citation</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>checksum_or_manifest</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>limitations</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>mirrors</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>verification_status</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>derived_status</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>verification_method</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>approx_size</t>
         </is>
@@ -48915,7 +49139,7 @@
       </c>
       <c r="AF88" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG88" t="inlineStr">
@@ -49092,7 +49316,7 @@
       </c>
       <c r="AF89" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG89" t="inlineStr">
@@ -50154,7 +50378,7 @@
       </c>
       <c r="AF95" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG95" t="inlineStr">
@@ -54260,42 +54484,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>repository</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>programmatic_access</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>access_model</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>search_method</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>container_reachable_2026_10_04</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>datasets_in_catalogue</t>
         </is>

</xml_diff>

<commit_message>
Acquire and validate PhysioNet batch-2 sets; catch silently truncated downloads
TS-002 (PTB-XL), TS-004 (Challenge 2017 AF), TS-006 (EEG motor imagery)
and TS-014 (Apnea-ECG) are downloaded and validated: checksums match the
shipped SHA256SUMS where present, and the waveforms parse.

The first attempt at the three large zips was cut at ~1.1 GB with a clean
end of stream, which the downloader logged as success. It now compares the
bytes received with Content-Length/Content-Range and resumes if short. Those
three manifest rows are corrected to failed.

The validator now finds WFDB records in a nested training*.zip, reads EDF
archives with wfdb, and skips macOS resource-fork files.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01233dsRAwyA6Arys3vibR2G
</commit_message>
<xml_diff>
--- a/healthcare-datasets/catalog/master_catalog.xlsx
+++ b/healthcare-datasets/catalog/master_catalog.xlsx
@@ -33,7 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Source registry'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Access restrictions'!$A$1:$H$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'QML feasibility'!$A$1:$W$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Acquisition manifest'!$A$1:$M$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Acquisition manifest'!$A$1:$M$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Overlaps &amp; mirrors'!$A$1:$C$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11140,7 +11140,7 @@
       </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T100" t="inlineStr">
@@ -11354,7 +11354,7 @@
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -12424,7 +12424,7 @@
       </c>
       <c r="S112" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T112" t="inlineStr">
@@ -16177,7 +16177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:M64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19305,8 +19305,419 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>TS-014</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/apnea-ecg/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>apnea_ecg_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>time_series/sleep/raw/TS-014/apnea_ecg_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:41:32Z</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>608841016</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>98681529dc9e795573cf28a158c289d20ed6cdcc95c9a23479c19282d8a4ec52</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>TS-004</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/challenge-2017/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>challenge_2017_af.zip</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>time_series/ecg/raw/TS-004/challenge_2017_af.zip</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:41:29Z</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>1206779393</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>17e964d8727ed87f1ded571686a6db2454eb83050aa552493302f63f54a5b041</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Truncated: stream ended at 1206779393 of 1476206149 bytes without an error (found 2026-10-04; downloader now checks size and resumes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>TS-002</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/ptb-xl/get-zip/1.0.3/</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ptb_xl_1.0.3.zip</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>time_series/ecg/raw/TS-002/ptb_xl_1.0.3.zip</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:41:35Z</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>1.0.3 (latest, published 2022-11-09)</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>1172569692</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>e4a841f7ea839c3c9149dfd70d2c7f796685320c4fd0f1a139ae9b835394a98f</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Truncated: stream ended at 1172569692 of 1839504686 bytes without an error (found 2026-10-04; downloader now checks size and resumes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>TS-006</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/eegmmidb/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>eegmmidb_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>time_series/eeg/raw/TS-006/eegmmidb_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:41:38Z</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>1175371384</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>628e72067b45889d85d1605aa20eb023da56d132f438ec08fa6fb549998c67c6</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>Truncated: stream ended at 1175371384 of 1997435063 bytes without an error (found 2026-10-04; downloader now checks size and resumes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>TS-004</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/challenge-2017/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>challenge_2017_af.zip</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>time_series/ecg/raw/TS-004/challenge_2017_af.zip</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2026-10-04T17:56:21Z</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
+        <v>1476206149</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>6cd773b2a4f5d94477e6c2541aa3f75497517d4d6cba3ac58353c6d2059a1723</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>TS-002</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/ptb-xl/get-zip/1.0.3/</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ptb_xl_1.0.3.zip</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>time_series/ecg/raw/TS-002/ptb_xl_1.0.3.zip</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>2026-10-04T17:56:24Z</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>1.0.3 (latest, published 2022-11-09)</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>1839504686</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>2d98687a9c69c8df03dbd69e0c569b3363981a0f667861c279c747d4aec29812</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>TS-006</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://www.physionet.org/content/eegmmidb/get-zip/1.0.0/</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>None; must conform to license terms (PhysioNet open access)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>eegmmidb_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>time_series/eeg/raw/TS-006/eegmmidb_1.0.0.zip</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>2026-10-04T17:56:27Z</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>1997435063</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>0ff5f7f38d1d14b8e485581ad4cf5b327e6494bc2ac7c7d7d4f7e9518a950cbe</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M57"/>
+  <autoFilter ref="A1:M64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27266,7 +27677,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -27480,7 +27891,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -27694,7 +28105,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -28550,7 +28961,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -50998,7 +51409,7 @@
       </c>
       <c r="AF100" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG100" t="inlineStr">
@@ -51352,7 +51763,7 @@
       </c>
       <c r="AF102" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG102" t="inlineStr">
@@ -51706,7 +52117,7 @@
       </c>
       <c r="AF104" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG104" t="inlineStr">
@@ -53122,7 +53533,7 @@
       </c>
       <c r="AF112" t="inlineStr">
         <is>
-          <t>Access verified</t>
+          <t>Parsed</t>
         </is>
       </c>
       <c r="AG112" t="inlineStr">

</xml_diff>